<commit_message>
feat: Demo D2 - Movement 输入解耦 + ChargeAI Sa 化 + Hero 蓝立方体
- §5.1 Movement 退化为纯执行器, 只读 MovementInfo.dire/wantmove
- 新增 Pilot Behavior, 玩家侧把 Gamepad 翻译成 MovementInfo
- 新增 Sa.ChargeAI System 型 Behavior (挂 Stage Actor), 每帧只收集一次 Hero 位置, 遍历所有 ChargeAIInfo 写对应 MovementInfo, 复杂度从 O(enemy×hero) 降到 O(enemy+hero)
- ChargeAIInfo 保留在常规 BehaviorInfos 下, 持有 attackrange/target
- EnemyPrefab 只挂 ChargeAIInfo (attackrange 来自 EnemyData.AttackRange mm→FP), 不再挂 Behavior
- TICK_DEFINE 时序补 Pilot / ChargeAI (都在 Movement 之前)
- EnemyData.xlsx 新增 AttackRange 列 + Luban 重生成
- HeroData Model 改指向 CubeBlue (蓝色立方体, 方便看朝向)
- DEMO_PLAN 同步 D2 完成清单与决策记录
</commit_message>
<xml_diff>
--- a/Config/Datas/EnemyData.xlsx
+++ b/Config/Datas/EnemyData.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
@@ -535,6 +535,11 @@
           <t>DeathPipelines</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>AttackRange</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -582,6 +587,11 @@
           <t>(list#sep=|),int</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -627,6 +637,11 @@
       <c r="I3" s="7" t="inlineStr">
         <is>
           <t>死亡管线</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>攻击距离(毫米)</t>
         </is>
       </c>
     </row>
@@ -650,6 +665,9 @@
       </c>
       <c r="I4" s="0" t="n">
         <v>10010</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: 还债 T1/T2 + Born Pipeline 补全
T1 Stage.cs: 删除临时强制切 IDLE 和测试 Buff
T2 BulletPrefab: model 字段由调用方传入，删除硬编码 200001
Born Pipeline: 新增 S10000（通用出生，切 IDLE），Hero/Enemy BornPipelines 填入 10000

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Config/Datas/EnemyData.xlsx
+++ b/Config/Datas/EnemyData.xlsx
@@ -535,7 +535,7 @@
           <t>DeathPipelines</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="0" t="inlineStr">
         <is>
           <t>AttackRange</t>
         </is>
@@ -587,7 +587,7 @@
           <t>(list#sep=|),int</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="0" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -639,7 +639,7 @@
           <t>死亡管线</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="0" t="inlineStr">
         <is>
           <t>攻击距离(毫米)</t>
         </is>
@@ -663,10 +663,13 @@
       <c r="F4" s="0" t="n">
         <v>10001</v>
       </c>
+      <c r="H4" t="n">
+        <v>10000</v>
+      </c>
       <c r="I4" s="0" t="n">
         <v>10010</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="0" t="n">
         <v>1500</v>
       </c>
     </row>

</xml_diff>